<commit_message>
add structured latency and retrieval logging across pipeline nodes
</commit_message>
<xml_diff>
--- a/src/data_processing/patient_kb/conversations/mayo_clinic_patient_clinician_dialogues.xlsx
+++ b/src/data_processing/patient_kb/conversations/mayo_clinic_patient_clinician_dialogues.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gahyunyoon/Desktop/classes/capstone/mayo-clinic-chatbot/src/data_processing/patient_kb/conversations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A33BEF1-3E1B-AA49-B53A-B2FB5C3FE382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9B9577-C200-F443-ADD0-D720A97AFD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conversations" sheetId="1" r:id="rId1"/>
@@ -5636,11 +5636,11 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5979,10 +5979,10 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="8" t="s">
         <v>1826</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -6032,7 +6032,7 @@
       <c r="F3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -7274,7 +7274,7 @@
       <c r="F49" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="G49" s="2" t="s">
+      <c r="G49" s="7" t="s">
         <v>121</v>
       </c>
       <c r="H49" s="2" t="s">
@@ -29602,11 +29602,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>1771</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">

</xml_diff>